<commit_message>
addition of medtronic handling in cleanCGM with additions made to the cgm dictionary
</commit_message>
<xml_diff>
--- a/inst/extdata/cgmvariable_dictionary.xlsx
+++ b/inst/extdata/cgmvariable_dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alicecarr/Desktop/CGMprocessing/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{406F0CC3-9AC9-764C-9783-914959BBE30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9912EBE5-93EC-8247-BD78-56112B26F0B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="37460" yWindow="3000" windowWidth="20360" windowHeight="12040" xr2:uid="{95CED60D-52FF-9E44-B892-971B4CE0580C}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15880" xr2:uid="{95CED60D-52FF-9E44-B892-971B4CE0580C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="31">
   <si>
     <t>old_vars</t>
   </si>
@@ -108,6 +108,30 @@
   </si>
   <si>
     <t>Historic Glucose mmol/L</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>CGM Glucose Value (mmol/l)</t>
+  </si>
+  <si>
+    <t>medtronic</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>medtronic_date</t>
+  </si>
+  <si>
+    <t>medtronic_time</t>
+  </si>
+  <si>
+    <t>Sensor Glucose (mmol/L)</t>
   </si>
 </sst>
 </file>
@@ -472,10 +496,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4196811C-C02D-BF4D-A15B-96DBE2D70C76}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
@@ -658,6 +683,90 @@
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
     </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>